<commit_message>
feat: 增加多种密度分布测量方式（CPU2 V0.12.0.0 / CPU3 V0.15.0.0）
版本：
- CPU2：V0.12.0.0（历史提交编号）
- CPU3：V0.15.0.0（历史提交编号）

协议版本/兼容性：
- 涉及 CPU2/CPU3 内部通信或寄存器映射；地址和字段口径以该历史提交的代码树为准。

本次修改：
- 增加普通分布、国标、每米和区间密度测量。
- 统一测点生成、单点采样、结果汇总和 CPU3 结果读取。

验证：
- 提交差异复核：通过；本次仅重写说明，代码树保持不变。
</commit_message>
<xml_diff>
--- a/LTD_MAIN_CPU2/docs/LTD故障代码表.xlsx
+++ b/LTD_MAIN_CPU2/docs/LTD故障代码表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="32565" windowHeight="17655"/>
+    <workbookView windowHeight="17655" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="总表" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="369">
   <si>
     <t>故障类型</t>
   </si>
@@ -796,6 +796,12 @@
     <t>数据校验</t>
   </si>
   <si>
+    <t>分布测量上限</t>
+  </si>
+  <si>
+    <t>分布测量下限</t>
+  </si>
+  <si>
     <t>结构体</t>
   </si>
   <si>
@@ -1127,6 +1133,9 @@
   </si>
   <si>
     <t>密度分布测量数据</t>
+  </si>
+  <si>
+    <t>数据更新标志位</t>
   </si>
 </sst>
 </file>
@@ -2404,7 +2413,7 @@
       <c r="P1" s="8"/>
       <c r="Q1" s="8"/>
     </row>
-    <row r="2" spans="4:17">
+    <row r="2" spans="2:17">
       <c r="D2" s="8"/>
       <c r="H2">
         <v>1</v>
@@ -2437,7 +2446,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="2:6">
+    <row r="3" spans="2:17">
       <c r="B3" s="8" t="s">
         <v>6</v>
       </c>
@@ -2454,7 +2463,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:6">
+    <row r="4" spans="2:17">
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
       <c r="D4" s="8">
@@ -2467,7 +2476,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="2:6">
+    <row r="5" spans="2:17">
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8">
@@ -2480,7 +2489,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:6">
+    <row r="6" spans="2:17">
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
       <c r="D6" s="8">
@@ -2493,7 +2502,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="2:6">
+    <row r="7" spans="2:17">
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
       <c r="D7" s="8">
@@ -2506,7 +2515,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="2:6">
+    <row r="8" spans="2:17">
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8">
@@ -2519,7 +2528,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="2:6">
+    <row r="9" spans="2:17">
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
       <c r="D9" s="8">
@@ -2532,7 +2541,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="2:6">
+    <row r="10" spans="2:17">
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
       <c r="D10" s="8">
@@ -2545,7 +2554,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="2:6">
+    <row r="11" spans="2:17">
       <c r="B11" s="8" t="s">
         <v>23</v>
       </c>
@@ -2562,7 +2571,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="2:6">
+    <row r="12" spans="2:17">
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
       <c r="D12" s="8">
@@ -2575,7 +2584,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="2:6">
+    <row r="13" spans="2:17">
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
       <c r="D13" s="8">
@@ -2588,7 +2597,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="2:6">
+    <row r="14" spans="2:17">
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
       <c r="D14" s="8">
@@ -2601,7 +2610,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="2:6">
+    <row r="15" spans="2:17">
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
       <c r="D15" s="8">
@@ -2614,7 +2623,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="2:6">
+    <row r="16" spans="2:17">
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
       <c r="D16" s="8">
@@ -3119,16 +3128,16 @@
         <v>112</v>
       </c>
     </row>
-    <row r="53" spans="4:4">
+    <row r="53" spans="2:6">
       <c r="D53" s="8"/>
     </row>
-    <row r="54" spans="4:4">
+    <row r="54" spans="2:6">
       <c r="D54" s="8"/>
     </row>
-    <row r="55" spans="4:4">
+    <row r="55" spans="2:6">
       <c r="D55" s="8"/>
     </row>
-    <row r="56" spans="4:4">
+    <row r="56" spans="2:6">
       <c r="D56" s="8"/>
     </row>
   </sheetData>
@@ -3180,7 +3189,7 @@
     <col min="4" max="4" width="35.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="18.75" spans="1:1">
+    <row r="2" ht="18.75" spans="1:4">
       <c r="A2" s="3" t="s">
         <v>113</v>
       </c>
@@ -3298,7 +3307,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="13" ht="18.75" spans="1:1">
+    <row r="13" ht="18.75" spans="1:4">
       <c r="A13" s="3" t="s">
         <v>141</v>
       </c>
@@ -3374,7 +3383,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="21" ht="18.75" spans="1:1">
+    <row r="21" ht="18.75" spans="1:4">
       <c r="A21" s="3" t="s">
         <v>154</v>
       </c>
@@ -3408,7 +3417,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" ht="18.75" spans="1:1">
+    <row r="26" ht="18.75" spans="1:4">
       <c r="A26" s="3" t="s">
         <v>158</v>
       </c>
@@ -3456,7 +3465,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="32" ht="18.75" spans="1:1">
+    <row r="32" ht="18.75" spans="1:4">
       <c r="A32" s="3" t="s">
         <v>165</v>
       </c>
@@ -3616,7 +3625,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="46" ht="18.75" spans="1:1">
+    <row r="46" ht="18.75" spans="1:4">
       <c r="A46" s="3" t="s">
         <v>194</v>
       </c>
@@ -3664,7 +3673,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="52" ht="18.75" spans="1:1">
+    <row r="52" ht="18.75" spans="1:4">
       <c r="A52" s="3" t="s">
         <v>201</v>
       </c>
@@ -3740,7 +3749,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="60" ht="18.75" spans="1:1">
+    <row r="60" ht="18.75" spans="1:4">
       <c r="A60" s="3" t="s">
         <v>213</v>
       </c>
@@ -3788,7 +3797,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="66" ht="18.75" spans="1:1">
+    <row r="66" ht="18.75" spans="1:4">
       <c r="A66" s="3" t="s">
         <v>220</v>
       </c>
@@ -3836,7 +3845,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="72" ht="18.75" spans="1:1">
+    <row r="72" ht="18.75" spans="1:4">
       <c r="A72" s="3" t="s">
         <v>226</v>
       </c>
@@ -3982,7 +3991,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="85" ht="18.75" spans="1:1">
+    <row r="85" ht="18.75" spans="1:4">
       <c r="A85" s="3" t="s">
         <v>251</v>
       </c>
@@ -4016,11 +4025,18 @@
         <v>254</v>
       </c>
     </row>
-    <row r="90" ht="22.5" spans="1:1">
+    <row r="90" ht="22.5" spans="1:4">
       <c r="A90" s="6"/>
     </row>
-    <row r="95" spans="1:1">
-      <c r="A95" s="7"/>
+    <row r="95" spans="1:4">
+      <c r="A95" s="7" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4">
+      <c r="A96" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="97" spans="1:1">
       <c r="A97" s="7"/>
@@ -4046,7 +4062,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="26" style="1" customWidth="1"/>
@@ -4058,66 +4074,66 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:4">
       <c r="A1" s="2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" s="1" customFormat="1" spans="1:4">
       <c r="A2" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" s="1" customFormat="1" spans="1:4">
       <c r="A3" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="1" spans="1:4">
       <c r="A4" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="1" spans="1:4">
       <c r="A5" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>119</v>
@@ -4128,374 +4144,374 @@
     </row>
     <row r="6" s="1" customFormat="1" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="1" spans="1:4">
       <c r="A7" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="1" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" s="1" customFormat="1" spans="1:4">
       <c r="A9" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" s="1" customFormat="1" spans="1:4">
       <c r="A10" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="11" s="1" customFormat="1" spans="1:4">
       <c r="A11" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="12" s="1" customFormat="1" spans="1:4">
       <c r="A12" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13" s="1" customFormat="1" spans="1:4">
       <c r="A13" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" spans="1:4">
       <c r="A14" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="15" s="1" customFormat="1" spans="1:4">
       <c r="A15" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="16" s="1" customFormat="1" spans="1:4">
       <c r="A16" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="17" s="1" customFormat="1" spans="1:4">
       <c r="A17" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="18" s="1" customFormat="1" spans="1:4">
       <c r="A18" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="19" s="1" customFormat="1" spans="1:4">
       <c r="A19" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="20" s="1" customFormat="1" spans="1:4">
       <c r="A20" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" spans="1:4">
       <c r="A21" s="1" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="22" s="1" customFormat="1" spans="1:4">
       <c r="A22" s="1" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="23" s="1" customFormat="1" spans="1:4">
       <c r="A23" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="24" s="1" customFormat="1" spans="1:4">
       <c r="A24" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>309</v>
-      </c>
       <c r="D24" s="1" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="25" s="1" customFormat="1" spans="1:4">
       <c r="A25" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="26" s="1" customFormat="1" spans="1:4">
       <c r="A26" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="27" s="1" customFormat="1" spans="1:4">
       <c r="A27" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" spans="1:4">
       <c r="A28" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="29" s="1" customFormat="1" spans="1:4">
       <c r="A29" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="30" s="1" customFormat="1" spans="1:4">
       <c r="A30" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="31" s="1" customFormat="1" spans="1:4">
       <c r="A31" s="1" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="32" s="1" customFormat="1" spans="1:4">
       <c r="A32" s="1" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>123</v>
@@ -4506,254 +4522,259 @@
     </row>
     <row r="33" s="1" customFormat="1" spans="1:4">
       <c r="A33" s="1" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="34" s="1" customFormat="1" spans="1:4">
       <c r="A34" s="1" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" spans="1:4">
       <c r="A35" s="1" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="36" s="1" customFormat="1" spans="1:4">
       <c r="A36" s="1" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="37" s="1" customFormat="1" spans="1:4">
       <c r="A37" s="1" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="38" s="1" customFormat="1" spans="1:4">
       <c r="A38" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="39" s="1" customFormat="1" spans="1:4">
       <c r="A39" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="40" s="1" customFormat="1" spans="1:4">
       <c r="A40" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B40" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>341</v>
-      </c>
       <c r="D40" s="1" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="41" s="1" customFormat="1" spans="1:4">
       <c r="A41" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="42" s="1" customFormat="1" spans="1:4">
       <c r="A42" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="43" s="1" customFormat="1" spans="1:4">
       <c r="A43" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="44" s="1" customFormat="1" spans="1:4">
       <c r="A44" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="45" s="1" customFormat="1" spans="1:4">
       <c r="A45" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="46" s="1" customFormat="1" spans="1:4">
       <c r="A46" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="47" s="1" customFormat="1" spans="1:4">
       <c r="A47" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="48" s="1" customFormat="1" spans="1:4">
       <c r="A48" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="49" s="1" customFormat="1" spans="1:4">
       <c r="A49" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="50" s="1" customFormat="1" spans="1:4">
       <c r="A50" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>365</v>
+        <v>367</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="1" t="s">
+        <v>368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: 修正CPU3本机参数被重复同步的问题（CPU2 V0.14.2.0 / CPU3 V0.15.1.0）
版本：
- CPU2：V0.14.2.0（历史提交编号）
- CPU3：V0.15.1.0（历史提交编号）

协议版本/兼容性：
- 涉及 CPU2/CPU3 内部通信或寄存器映射；地址和字段口径以该历史提交的代码树为准。

本次修改：
- CPU3 批量同步参数时跳过本机参数，避免配置错位。
- 补充罐底状态检查并移除临时锁文件。

验证：
- 提交差异复核：通过；本次仅重写说明，代码树保持不变。
</commit_message>
<xml_diff>
--- a/LTD_MAIN_CPU2/docs/LTD故障代码表.xlsx
+++ b/LTD_MAIN_CPU2/docs/LTD故障代码表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17655" activeTab="2"/>
+    <workbookView windowWidth="32745" windowHeight="17655" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="总表" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="386">
   <si>
     <t>故障类型</t>
   </si>
@@ -1158,6 +1158,15 @@
   </si>
   <si>
     <t>水位罐高</t>
+  </si>
+  <si>
+    <t>水位电容阈值</t>
+  </si>
+  <si>
+    <t>水位滞后阈</t>
+  </si>
+  <si>
+    <t>水位标定值</t>
   </si>
   <si>
     <t>电机步进数</t>
@@ -4854,6 +4863,15 @@
       <c r="A61" s="1" t="s">
         <v>375</v>
       </c>
+      <c r="B61" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>378</v>
+      </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="3" t="s">
@@ -4867,37 +4885,37 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="1" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
     </row>
     <row r="65" spans="1:1">
       <c r="A65" s="1" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="66" spans="1:1">
       <c r="A66" s="1" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="67" spans="1:1">
       <c r="A67" s="1" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
     </row>
     <row r="68" spans="1:1">
       <c r="A68" s="1" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
     </row>
     <row r="69" spans="1:1">
       <c r="A69" s="1" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
     </row>
     <row r="70" spans="1:1">
       <c r="A70" s="1" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>

</xml_diff>